<commit_message>
aggiunti manualmente i link che usati dallo scraper di booking
</commit_message>
<xml_diff>
--- a/datasets/availability_dataset_2022-09-17_2022-09-24_booking.xlsx
+++ b/datasets/availability_dataset_2022-09-17_2022-09-24_booking.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G133"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -466,7 +466,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Camera Matrimoniale con Terrazza</t>
+          <t>Chalet con 1 Camera da Letto - Servizio Alberghiero e Servizio Spiaggia Inclusi</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -474,22 +474,22 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>€ 368</t>
+          <t>€ 1.204</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>€ 338</t>
+          <t>€ 1.034</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/nuovo-natural-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>camping-village-mar-y-sierra</t>
+          <t>nuovo-natural-village</t>
         </is>
       </c>
     </row>
@@ -499,30 +499,30 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Bungalow con 1 Camera da Letto</t>
+          <t>Chalet con 1 Camera da Letto - Servizio Alberghiero e Servizio Spiaggia Inclusi</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>€ 423</t>
+          <t>€ 1.799</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>€ 393</t>
+          <t>€ 1.544</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/nuovo-natural-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>camping-village-mar-y-sierra</t>
+          <t>nuovo-natural-village</t>
         </is>
       </c>
     </row>
@@ -532,30 +532,30 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Chalet</t>
+          <t>Chalet con 1 Camera da Letto - Servizio Alberghiero e Servizio Spiaggia Inclusi</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>€ 423</t>
+          <t>€ 602</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>€ 393</t>
+          <t>€ 517</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/nuovo-natural-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>camping-village-mar-y-sierra</t>
+          <t>nuovo-natural-village</t>
         </is>
       </c>
     </row>
@@ -565,30 +565,30 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Bungalow con 2 Camere da Letto</t>
+          <t>Chalet con 2 Camere da Letto - Servizio Alberghiero e Servizio Spiaggia Inclusi</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>€ 459</t>
+          <t>€ 1.204</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>€ 427</t>
+          <t>€ 1.034</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/nuovo-natural-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>camping-village-mar-y-sierra</t>
+          <t>nuovo-natural-village</t>
         </is>
       </c>
     </row>
@@ -598,30 +598,30 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Villa con 2 Camere da Letto</t>
+          <t>Chalet con 2 Camere da Letto - Servizio Alberghiero e Servizio Spiaggia Inclusi</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>€ 496</t>
+          <t>€ 1.799</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>€ 461</t>
+          <t>€ 1.544</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/nuovo-natural-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>camping-village-mar-y-sierra</t>
+          <t>nuovo-natural-village</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Camera Quadrupla</t>
+          <t>Chalet con 2 Camere da Letto - Servizio Alberghiero e Servizio Spiaggia Inclusi</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -639,22 +639,22 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>€ 515</t>
+          <t>€ 2.394</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>€ 473</t>
+          <t>€ 2.054</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/nuovo-natural-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>camping-village-mar-y-sierra</t>
+          <t>nuovo-natural-village</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tenda</t>
+          <t>Chalet con 2 Camere da Letto - Servizio Alberghiero e Servizio Spiaggia Inclusi</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -672,22 +672,22 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>€ 423</t>
+          <t>€ 2.989</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>€ 393</t>
+          <t>€ 2.564</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/nuovo-natural-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>camping-village-mar-y-sierra</t>
+          <t>nuovo-natural-village</t>
         </is>
       </c>
     </row>
@@ -697,26 +697,30 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Bungalow</t>
+          <t>Chalet con 2 Camere da Letto - Servizio Alberghiero e Servizio Spiaggia Inclusi</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>3</v>
-      </c>
-      <c r="D9" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>€ 602</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>€ 371</t>
+          <t>€ 517</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/camping-la-pineta.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/nuovo-natural-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>camping-la-pineta</t>
+          <t>nuovo-natural-village</t>
         </is>
       </c>
     </row>
@@ -726,26 +730,26 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bungalow</t>
+          <t>Chalet con 1 Camera da Letto</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
-          <t>€ 1.162</t>
+          <t>€ 1.022</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/camping-la-pineta.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/nuovo-natural-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>camping-la-pineta</t>
+          <t>nuovo-natural-village</t>
         </is>
       </c>
     </row>
@@ -755,30 +759,30 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Chalet Superior con 1 Camera da Letto</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>€ 560</t>
+          <t>€ 994</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>€ 438</t>
+          <t>€ 854</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/nuovo-natural-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>nuovo-natural-village</t>
         </is>
       </c>
     </row>
@@ -788,30 +792,30 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Chalet con 2 Camere da Letto</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>€ 700</t>
+          <t>€ 1.064</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>€ 547</t>
+          <t>€ 914</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/nuovo-natural-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>nuovo-natural-village</t>
         </is>
       </c>
     </row>
@@ -821,30 +825,30 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Chalet Superior con 2 Camere da Letto</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>€ 840</t>
+          <t>€ 1.344</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 1.154</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/nuovo-natural-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>nuovo-natural-village</t>
         </is>
       </c>
     </row>
@@ -854,30 +858,26 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Tenda</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>€ 420</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>€ 328</t>
+          <t>€ 193</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -893,24 +893,20 @@
       <c r="C15" t="n">
         <v>2</v>
       </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>€ 560</t>
-        </is>
-      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>€ 438</t>
+          <t>€ 305</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -926,24 +922,20 @@
       <c r="C16" t="n">
         <v>3</v>
       </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>€ 700</t>
-        </is>
-      </c>
+      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
-          <t>€ 547</t>
+          <t>€ 263</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -957,26 +949,22 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>4</v>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>€ 840</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 431</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -990,26 +978,22 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>€ 420</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>€ 328</t>
+          <t>€ 333</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1023,26 +1007,22 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2</v>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>€ 560</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
-          <t>€ 438</t>
+          <t>€ 557</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1052,30 +1032,26 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Tenda</t>
+          <t>Casa Mobile Classic</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>3</v>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>€ 700</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
-          <t>€ 547</t>
+          <t>€ 208</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1085,30 +1061,26 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Tenda</t>
+          <t>Casa Mobile Classic</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>€ 840</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 320</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1118,30 +1090,26 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Tenda</t>
+          <t>Casa Mobile Classic</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>€ 420</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
-          <t>€ 328</t>
+          <t>€ 278</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1151,30 +1119,26 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Tenda</t>
+          <t>Casa Mobile Classic</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2</v>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>€ 560</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
-          <t>€ 438</t>
+          <t>€ 446</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1184,30 +1148,26 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tenda</t>
+          <t>Casa Mobile Classic</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>€ 700</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
-          <t>€ 547</t>
+          <t>€ 348</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1217,30 +1177,26 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Tenda</t>
+          <t>Casa Mobile Classic</t>
         </is>
       </c>
       <c r="C25" t="n">
         <v>4</v>
       </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>€ 840</t>
-        </is>
-      </c>
+      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 572</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1250,30 +1206,26 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Tenda</t>
+          <t>Chalet</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1</v>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>€ 420</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
-          <t>€ 328</t>
+          <t>€ 418</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1283,30 +1235,26 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Tenda</t>
+          <t>Chalet</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2</v>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>€ 560</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
-          <t>€ 438</t>
+          <t>€ 642</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1316,30 +1264,26 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Tenda</t>
+          <t>Chalet</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>3</v>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>€ 700</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
-          <t>€ 547</t>
+          <t>€ 488</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1349,30 +1293,26 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Tenda</t>
+          <t>Chalet</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>4</v>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>€ 840</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 768</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1382,30 +1322,26 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Tenda</t>
+          <t>Casa Mobile Deluxe</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>€ 420</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
-          <t>€ 328</t>
+          <t>€ 483</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1415,30 +1351,26 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Deluxe</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2</v>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>€ 560</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
-          <t>€ 438</t>
+          <t>€ 707</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1448,30 +1380,26 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Deluxe</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>3</v>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>€ 700</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
-          <t>€ 547</t>
+          <t>€ 553</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1481,30 +1409,26 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Deluxe</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>4</v>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>€ 840</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 833</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1514,30 +1438,26 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Deluxe - Fronte Mare</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1</v>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>€ 420</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
-          <t>€ 328</t>
+          <t>€ 558</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1547,30 +1467,26 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Deluxe - Fronte Mare</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>€ 560</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
-          <t>€ 438</t>
+          <t>€ 782</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1580,30 +1496,26 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Superior Fronte Mare</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>€ 700</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
-          <t>€ 547</t>
+          <t>€ 663</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1613,30 +1525,26 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Superior Fronte Mare</t>
         </is>
       </c>
       <c r="C37" t="n">
         <v>4</v>
       </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>€ 840</t>
-        </is>
-      </c>
+      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 887</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1646,30 +1554,26 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Superior Fronte Mare</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>€ 420</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
-          <t>€ 328</t>
+          <t>€ 733</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1679,30 +1583,26 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Superior Fronte Mare</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>€ 560</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
-          <t>€ 438</t>
+          <t>€ 957</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1712,30 +1612,26 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Tenda Superior</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3</v>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>€ 700</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
-          <t>€ 547</t>
+          <t>€ 1.043</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1745,30 +1641,26 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Tenda Superior</t>
         </is>
       </c>
       <c r="C41" t="n">
         <v>4</v>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>€ 840</t>
-        </is>
-      </c>
+      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 1.267</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1778,30 +1670,26 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Tenda Superior</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>€ 420</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr">
         <is>
-          <t>€ 328</t>
+          <t>€ 1.113</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1811,30 +1699,26 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Tenda Superior</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2</v>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>€ 560</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr">
         <is>
-          <t>€ 438</t>
+          <t>€ 1.393</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1844,30 +1728,26 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Tenda Superior</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>3</v>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>€ 700</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr">
         <is>
-          <t>€ 547</t>
+          <t>€ 1.183</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1877,30 +1757,26 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Tenda Superior</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>4</v>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>€ 840</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 1.519</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/girasole-camping-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>girasole-camping-village</t>
         </is>
       </c>
     </row>
@@ -1910,30 +1786,30 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Piccola</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>€ 420</t>
+          <t>€ 711</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>€ 328</t>
+          <t>€ 670</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/green-garden-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>green-garden-village</t>
         </is>
       </c>
     </row>
@@ -1943,30 +1819,26 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Piccola</t>
         </is>
       </c>
       <c r="C47" t="n">
         <v>2</v>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>€ 560</t>
-        </is>
-      </c>
+      <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr">
         <is>
-          <t>€ 438</t>
+          <t>€ 711</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/green-garden-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>green-garden-village</t>
         </is>
       </c>
     </row>
@@ -1976,30 +1848,30 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Monolocale su 2 Livelli</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>€ 700</t>
+          <t>€ 651</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>€ 547</t>
+          <t>€ 603</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/green-garden-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>green-garden-village</t>
         </is>
       </c>
     </row>
@@ -2009,30 +1881,30 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Monolocale su 2 Livelli</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>€ 840</t>
+          <t>€ 791</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 732</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/green-garden-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>green-garden-village</t>
         </is>
       </c>
     </row>
@@ -2042,30 +1914,26 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Camera Matrimoniale</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1</v>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>€ 420</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>€ 328</t>
+          <t>€ 708</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/green-garden-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>green-garden-village</t>
         </is>
       </c>
     </row>
@@ -2075,30 +1943,26 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Camera Matrimoniale</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2</v>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>€ 560</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
-          <t>€ 438</t>
+          <t>€ 883</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/green-garden-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>green-garden-village</t>
         </is>
       </c>
     </row>
@@ -2108,30 +1972,30 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>€ 700</t>
+          <t>€ 901</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>€ 547</t>
+          <t>€ 845</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/green-garden-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>green-garden-village</t>
         </is>
       </c>
     </row>
@@ -2141,30 +2005,26 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile</t>
         </is>
       </c>
       <c r="C53" t="n">
         <v>4</v>
       </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>€ 840</t>
-        </is>
-      </c>
+      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 901</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/green-garden-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>green-garden-village</t>
         </is>
       </c>
     </row>
@@ -2174,30 +2034,30 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Luxury</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>€ 420</t>
+          <t>€ 991</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>€ 328</t>
+          <t>€ 913</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/green-garden-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>green-garden-village</t>
         </is>
       </c>
     </row>
@@ -2207,30 +2067,26 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Luxury</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2</v>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>€ 560</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr">
         <is>
-          <t>€ 438</t>
+          <t>€ 991</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/green-garden-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>green-garden-village</t>
         </is>
       </c>
     </row>
@@ -2240,30 +2096,30 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Luxury</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>€ 700</t>
+          <t>€ 1.131</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>€ 547</t>
+          <t>€ 1.042</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/green-garden-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>green-garden-village</t>
         </is>
       </c>
     </row>
@@ -2273,30 +2129,26 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile Luxury</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>4</v>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>€ 840</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 1.131</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/green-garden-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>green-garden-village</t>
         </is>
       </c>
     </row>
@@ -2306,30 +2158,30 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile (6 Adulti)</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>€ 420</t>
+          <t>€ 1.191</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>€ 328</t>
+          <t>€ 1.111</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/green-garden-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>green-garden-village</t>
         </is>
       </c>
     </row>
@@ -2339,30 +2191,26 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Casa Mobile (6 Adulti)</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2</v>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>€ 560</t>
-        </is>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr">
         <is>
-          <t>€ 438</t>
+          <t>€ 1.191</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/green-garden-village.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>green-garden-village</t>
         </is>
       </c>
     </row>
@@ -2372,30 +2220,30 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Camera Matrimoniale con Terrazza</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>€ 700</t>
+          <t>€ 368</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>€ 547</t>
+          <t>€ 349</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>camping-village-mar-y-sierra</t>
         </is>
       </c>
     </row>
@@ -2405,30 +2253,30 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Bungalow con 1 Camera da Letto</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>€ 840</t>
+          <t>€ 423</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 404</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>camping-village-mar-y-sierra</t>
         </is>
       </c>
     </row>
@@ -2438,30 +2286,30 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Chalet</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>€ 420</t>
+          <t>€ 423</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>€ 328</t>
+          <t>€ 404</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>camping-village-mar-y-sierra</t>
         </is>
       </c>
     </row>
@@ -2471,30 +2319,30 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Bungalow con 2 Camere da Letto</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>€ 560</t>
+          <t>€ 459</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>€ 438</t>
+          <t>€ 439</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>camping-village-mar-y-sierra</t>
         </is>
       </c>
     </row>
@@ -2504,30 +2352,30 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Villa con 2 Camere da Letto</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>€ 700</t>
+          <t>€ 496</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>€ 547</t>
+          <t>€ 474</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>camping-village-mar-y-sierra</t>
         </is>
       </c>
     </row>
@@ -2537,7 +2385,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Camera Quadrupla</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -2545,22 +2393,22 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>€ 840</t>
+          <t>€ 515</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 489</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>camping-village-mar-y-sierra</t>
         </is>
       </c>
     </row>
@@ -2570,30 +2418,30 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Piazzola</t>
+          <t>Tenda</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>€ 420</t>
+          <t>€ 423</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>€ 328</t>
+          <t>€ 404</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/camping-village-mar-y-sierra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>camping-village-mar-y-sierra</t>
         </is>
       </c>
     </row>
@@ -2603,30 +2451,30 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Tenda</t>
+          <t>Casa con 1 Camera da Letto</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>€ 840</t>
+          <t>€ 1.323</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 1.250</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/poggio-imperiale-marche-civitanova-marche-5.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>poggio-imperiale-marche-civitanova-marche-5</t>
         </is>
       </c>
     </row>
@@ -2636,30 +2484,26 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto</t>
+          <t>Casa con 1 Camera da Letto</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2</v>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>€ 1.400</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr">
         <is>
-          <t>€ 1.095</t>
+          <t>€ 1.470</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/poggio-imperiale-marche-civitanova-marche-5.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>poggio-imperiale-marche-civitanova-marche-5</t>
         </is>
       </c>
     </row>
@@ -2669,30 +2513,26 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto</t>
+          <t>Tenda</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>3</v>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>€ 1.575</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr">
         <is>
-          <t>€ 1.232</t>
+          <t>€ 700</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/agriturismo-la-viola-e-il-sole.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>agriturismo-la-viola-e-il-sole</t>
         </is>
       </c>
     </row>
@@ -2702,30 +2542,26 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto</t>
+          <t>Tenda</t>
         </is>
       </c>
       <c r="C70" t="n">
         <v>4</v>
       </c>
-      <c r="D70" t="inlineStr">
-        <is>
-          <t>€ 1.750</t>
-        </is>
-      </c>
+      <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr">
         <is>
-          <t>€ 1.369</t>
+          <t>€ 840</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/resort-orizzonti-glamping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>resort-orizzonti-glamping</t>
         </is>
       </c>
     </row>
@@ -2735,30 +2571,26 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto</t>
+          <t>Tenda</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1</v>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>€ 1.225</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr">
         <is>
-          <t>€ 958</t>
+          <t>€ 910</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/resort-orizzonti-glamping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>resort-orizzonti-glamping</t>
         </is>
       </c>
     </row>
@@ -2768,7 +2600,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto</t>
+          <t>Tenda</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -2776,22 +2608,22 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>€ 1.400</t>
+          <t>€ 464</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>€ 1.095</t>
+          <t>€ 434</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/glamping-marche-nascoste-tenda-e-intero-alloggio.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>glamping-marche-nascoste-tenda-e-intero-alloggio</t>
         </is>
       </c>
     </row>
@@ -2801,7 +2633,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto</t>
+          <t>Tenda</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -2809,22 +2641,22 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>€ 1.575</t>
+          <t>€ 618</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>€ 1.232</t>
+          <t>€ 578</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/glamping-marche-nascoste-tenda-e-intero-alloggio.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>glamping-marche-nascoste-tenda-e-intero-alloggio</t>
         </is>
       </c>
     </row>
@@ -2834,7 +2666,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto</t>
+          <t>Tenda</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -2842,22 +2674,22 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>€ 1.750</t>
+          <t>€ 464</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>€ 1.369</t>
+          <t>€ 434</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/glamping-marche-nascoste-tenda-e-intero-alloggio.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>glamping-marche-nascoste-tenda-e-intero-alloggio</t>
         </is>
       </c>
     </row>
@@ -2867,30 +2699,30 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto</t>
+          <t>Tenda</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>€ 1.225</t>
+          <t>€ 772</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>€ 958</t>
+          <t>€ 722</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/glamping-marche-nascoste-tenda-e-intero-alloggio.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>glamping-marche-nascoste-tenda-e-intero-alloggio</t>
         </is>
       </c>
     </row>
@@ -2900,30 +2732,30 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto</t>
+          <t>Tenda</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>€ 1.400</t>
+          <t>€ 429</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>€ 1.095</t>
+          <t>€ 401</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/glamping-marche-nascoste-tenda-e-intero-alloggio.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>glamping-marche-nascoste-tenda-e-intero-alloggio</t>
         </is>
       </c>
     </row>
@@ -2933,30 +2765,26 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto</t>
+          <t>Bungalow</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>3</v>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>€ 1.575</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr">
         <is>
-          <t>€ 1.232</t>
+          <t>€ 505</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/camping-pineta-urbino.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>camping-pineta-urbino</t>
         </is>
       </c>
     </row>
@@ -2966,30 +2794,26 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto</t>
+          <t>Bungalow</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>4</v>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>€ 1.750</t>
-        </is>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr">
         <is>
-          <t>€ 1.369</t>
+          <t>€ 724</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/camping-pineta-urbino.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>camping-pineta-urbino</t>
         </is>
       </c>
     </row>
@@ -2999,30 +2823,26 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto</t>
+          <t>Bungalow</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1</v>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>€ 1.225</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr">
         <is>
-          <t>€ 958</t>
+          <t>€ 942</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/camping-pineta-urbino.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>camping-pineta-urbino</t>
         </is>
       </c>
     </row>
@@ -3032,7 +2852,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto - Accesso Disabili</t>
+          <t>Camera Matrimoniale</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -3040,22 +2860,22 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>€ 1.400</t>
+          <t>€ 490</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>€ 1.095</t>
+          <t>€ 458</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/ai-due-camini.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>ai-due-camini</t>
         </is>
       </c>
     </row>
@@ -3065,30 +2885,30 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto - Accesso Disabili</t>
+          <t>Casa Mobile</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>€ 1.575</t>
+          <t>€ 748</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>€ 1.232</t>
+          <t>€ 692</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/amapolas-villaggio-amp-camping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>amapolas-villaggio-amp-camping</t>
         </is>
       </c>
     </row>
@@ -3098,30 +2918,30 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto - Accesso Disabili</t>
+          <t>Casa Mobile</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>€ 1.750</t>
+          <t>€ 1.273</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>€ 1.369</t>
+          <t>€ 1.175</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/amapolas-villaggio-amp-camping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>amapolas-villaggio-amp-camping</t>
         </is>
       </c>
     </row>
@@ -3131,30 +2951,30 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Appartamento con 1 Camera da Letto - Accesso Disabili</t>
+          <t>Casa Mobile</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>€ 1.225</t>
+          <t>€ 1.448</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>€ 958</t>
+          <t>€ 1.336</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/amapolas-villaggio-amp-camping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>amapolas-villaggio-amp-camping</t>
         </is>
       </c>
     </row>
@@ -3164,30 +2984,30 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Tenda</t>
+          <t>Casa Mobile</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>€ 840</t>
+          <t>€ 1.798</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>€ 657</t>
+          <t>€ 1.658</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/saecula.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/amapolas-villaggio-amp-camping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>saecula</t>
+          <t>amapolas-villaggio-amp-camping</t>
         </is>
       </c>
     </row>
@@ -3201,26 +3021,26 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>€ 407</t>
+          <t>€ 748</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>€ 378</t>
+          <t>€ 692</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/camping-terrazzo-sul-mare.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/amapolas-villaggio-amp-camping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>camping-terrazzo-sul-mare</t>
+          <t>amapolas-villaggio-amp-camping</t>
         </is>
       </c>
     </row>
@@ -3230,30 +3050,30 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Chalet con 2 Camere da Letto</t>
+          <t>Casa Mobile</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>€ 505</t>
+          <t>€ 1.168</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>€ 469</t>
+          <t>€ 1.078</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/camping-terrazzo-sul-mare.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/amapolas-villaggio-amp-camping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>camping-terrazzo-sul-mare</t>
+          <t>amapolas-villaggio-amp-camping</t>
         </is>
       </c>
     </row>
@@ -3263,30 +3083,30 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Roulotte</t>
+          <t>Casa Mobile</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>€ 413</t>
+          <t>€ 1.448</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>€ 380</t>
+          <t>€ 1.336</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/amapolas-villaggio-amp-camping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>parco-gessilandia</t>
+          <t>amapolas-villaggio-amp-camping</t>
         </is>
       </c>
     </row>
@@ -3296,30 +3116,30 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Roulotte</t>
+          <t>Camera Matrimoniale Deluxe</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>€ 553</t>
+          <t>€ 748</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>€ 509</t>
+          <t>€ 692</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/amapolas-villaggio-amp-camping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>parco-gessilandia</t>
+          <t>amapolas-villaggio-amp-camping</t>
         </is>
       </c>
     </row>
@@ -3329,30 +3149,30 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Roulotte</t>
+          <t>Camera Matrimoniale Deluxe</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>€ 693</t>
+          <t>€ 608</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>€ 638</t>
+          <t>€ 563</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/amapolas-villaggio-amp-camping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>parco-gessilandia</t>
+          <t>amapolas-villaggio-amp-camping</t>
         </is>
       </c>
     </row>
@@ -3362,30 +3182,30 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Roulotte</t>
+          <t>Casa Mobile</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>€ 763</t>
+          <t>€ 783</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>€ 702</t>
+          <t>€ 724</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/amapolas-villaggio-amp-camping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>parco-gessilandia</t>
+          <t>amapolas-villaggio-amp-camping</t>
         </is>
       </c>
     </row>
@@ -3395,30 +3215,30 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Roulotte</t>
+          <t>Casa Mobile</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>€ 833</t>
+          <t>€ 1.273</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>€ 766</t>
+          <t>€ 1.175</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/amapolas-villaggio-amp-camping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>parco-gessilandia</t>
+          <t>amapolas-villaggio-amp-camping</t>
         </is>
       </c>
     </row>
@@ -3428,30 +3248,30 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Roulotte</t>
+          <t>Bungalow con Vista Mare</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>€ 273</t>
+          <t>€ 1.124</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>€ 251</t>
+          <t>€ 1.040</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/bungalow-verde-mare.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>parco-gessilandia</t>
+          <t>bungalow-verde-mare</t>
         </is>
       </c>
     </row>
@@ -3461,30 +3281,26 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Roulotte</t>
+          <t>Bungalow con 2 Camere da Letto (4 Adulti)</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2</v>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>€ 413</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr">
         <is>
-          <t>€ 380</t>
+          <t>€ 680</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/camping-norina.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>parco-gessilandia</t>
+          <t>camping-norina</t>
         </is>
       </c>
     </row>
@@ -3494,1277 +3310,26 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Roulotte</t>
+          <t>Bungalow con 2 Camere da Letto (5 Adulti)</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>3</v>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>€ 553</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr">
         <is>
-          <t>€ 509</t>
+          <t>€ 785</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
+          <t>https://www.booking.com/hotel/it/camping-norina.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="1" t="n">
-        <v>93</v>
-      </c>
-      <c r="B95" t="inlineStr">
-        <is>
-          <t>Roulotte</t>
-        </is>
-      </c>
-      <c r="C95" t="n">
-        <v>4</v>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>€ 693</t>
-        </is>
-      </c>
-      <c r="E95" t="inlineStr">
-        <is>
-          <t>€ 638</t>
-        </is>
-      </c>
-      <c r="F95" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="1" t="n">
-        <v>94</v>
-      </c>
-      <c r="B96" t="inlineStr">
-        <is>
-          <t>Roulotte</t>
-        </is>
-      </c>
-      <c r="C96" t="n">
-        <v>5</v>
-      </c>
-      <c r="D96" t="inlineStr">
-        <is>
-          <t>€ 763</t>
-        </is>
-      </c>
-      <c r="E96" t="inlineStr">
-        <is>
-          <t>€ 702</t>
-        </is>
-      </c>
-      <c r="F96" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="1" t="n">
-        <v>95</v>
-      </c>
-      <c r="B97" t="inlineStr">
-        <is>
-          <t>Roulotte</t>
-        </is>
-      </c>
-      <c r="C97" t="n">
-        <v>6</v>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>€ 833</t>
-        </is>
-      </c>
-      <c r="E97" t="inlineStr">
-        <is>
-          <t>€ 766</t>
-        </is>
-      </c>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="1" t="n">
-        <v>96</v>
-      </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>Roulotte</t>
-        </is>
-      </c>
-      <c r="C98" t="n">
-        <v>1</v>
-      </c>
-      <c r="D98" t="inlineStr">
-        <is>
-          <t>€ 273</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>€ 251</t>
-        </is>
-      </c>
-      <c r="F98" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="1" t="n">
-        <v>97</v>
-      </c>
-      <c r="B99" t="inlineStr">
-        <is>
-          <t>Roulotte</t>
-        </is>
-      </c>
-      <c r="C99" t="n">
-        <v>2</v>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>€ 413</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>€ 380</t>
-        </is>
-      </c>
-      <c r="F99" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="1" t="n">
-        <v>98</v>
-      </c>
-      <c r="B100" t="inlineStr">
-        <is>
-          <t>Roulotte</t>
-        </is>
-      </c>
-      <c r="C100" t="n">
-        <v>3</v>
-      </c>
-      <c r="D100" t="inlineStr">
-        <is>
-          <t>€ 553</t>
-        </is>
-      </c>
-      <c r="E100" t="inlineStr">
-        <is>
-          <t>€ 509</t>
-        </is>
-      </c>
-      <c r="F100" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="1" t="n">
-        <v>99</v>
-      </c>
-      <c r="B101" t="inlineStr">
-        <is>
-          <t>Roulotte</t>
-        </is>
-      </c>
-      <c r="C101" t="n">
-        <v>4</v>
-      </c>
-      <c r="D101" t="inlineStr">
-        <is>
-          <t>€ 693</t>
-        </is>
-      </c>
-      <c r="E101" t="inlineStr">
-        <is>
-          <t>€ 638</t>
-        </is>
-      </c>
-      <c r="F101" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="1" t="n">
-        <v>100</v>
-      </c>
-      <c r="B102" t="inlineStr">
-        <is>
-          <t>Roulotte</t>
-        </is>
-      </c>
-      <c r="C102" t="n">
-        <v>5</v>
-      </c>
-      <c r="D102" t="inlineStr">
-        <is>
-          <t>€ 763</t>
-        </is>
-      </c>
-      <c r="E102" t="inlineStr">
-        <is>
-          <t>€ 702</t>
-        </is>
-      </c>
-      <c r="F102" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G102" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="1" t="n">
-        <v>101</v>
-      </c>
-      <c r="B103" t="inlineStr">
-        <is>
-          <t>Roulotte</t>
-        </is>
-      </c>
-      <c r="C103" t="n">
-        <v>1</v>
-      </c>
-      <c r="D103" t="inlineStr">
-        <is>
-          <t>€ 273</t>
-        </is>
-      </c>
-      <c r="E103" t="inlineStr">
-        <is>
-          <t>€ 251</t>
-        </is>
-      </c>
-      <c r="F103" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="1" t="n">
-        <v>102</v>
-      </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>Chalet</t>
-        </is>
-      </c>
-      <c r="C104" t="n">
-        <v>2</v>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>€ 553</t>
-        </is>
-      </c>
-      <c r="E104" t="inlineStr">
-        <is>
-          <t>€ 509</t>
-        </is>
-      </c>
-      <c r="F104" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="1" t="n">
-        <v>103</v>
-      </c>
-      <c r="B105" t="inlineStr">
-        <is>
-          <t>Chalet</t>
-        </is>
-      </c>
-      <c r="C105" t="n">
-        <v>3</v>
-      </c>
-      <c r="D105" t="inlineStr">
-        <is>
-          <t>€ 763</t>
-        </is>
-      </c>
-      <c r="E105" t="inlineStr">
-        <is>
-          <t>€ 702</t>
-        </is>
-      </c>
-      <c r="F105" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="1" t="n">
-        <v>104</v>
-      </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>Chalet</t>
-        </is>
-      </c>
-      <c r="C106" t="n">
-        <v>4</v>
-      </c>
-      <c r="D106" t="inlineStr">
-        <is>
-          <t>€ 903</t>
-        </is>
-      </c>
-      <c r="E106" t="inlineStr">
-        <is>
-          <t>€ 831</t>
-        </is>
-      </c>
-      <c r="F106" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="1" t="n">
-        <v>105</v>
-      </c>
-      <c r="B107" t="inlineStr">
-        <is>
-          <t>Chalet</t>
-        </is>
-      </c>
-      <c r="C107" t="n">
-        <v>5</v>
-      </c>
-      <c r="D107" t="inlineStr">
-        <is>
-          <t>€ 973</t>
-        </is>
-      </c>
-      <c r="E107" t="inlineStr">
-        <is>
-          <t>€ 895</t>
-        </is>
-      </c>
-      <c r="F107" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="1" t="n">
-        <v>106</v>
-      </c>
-      <c r="B108" t="inlineStr">
-        <is>
-          <t>Chalet</t>
-        </is>
-      </c>
-      <c r="C108" t="n">
-        <v>1</v>
-      </c>
-      <c r="D108" t="inlineStr">
-        <is>
-          <t>€ 343</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>€ 316</t>
-        </is>
-      </c>
-      <c r="F108" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="109">
-      <c r="A109" s="1" t="n">
-        <v>107</v>
-      </c>
-      <c r="B109" t="inlineStr">
-        <is>
-          <t>Chalet</t>
-        </is>
-      </c>
-      <c r="C109" t="n">
-        <v>2</v>
-      </c>
-      <c r="D109" t="inlineStr">
-        <is>
-          <t>€ 623</t>
-        </is>
-      </c>
-      <c r="E109" t="inlineStr">
-        <is>
-          <t>€ 573</t>
-        </is>
-      </c>
-      <c r="F109" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="110">
-      <c r="A110" s="1" t="n">
-        <v>108</v>
-      </c>
-      <c r="B110" t="inlineStr">
-        <is>
-          <t>Chalet</t>
-        </is>
-      </c>
-      <c r="C110" t="n">
-        <v>3</v>
-      </c>
-      <c r="D110" t="inlineStr">
-        <is>
-          <t>€ 833</t>
-        </is>
-      </c>
-      <c r="E110" t="inlineStr">
-        <is>
-          <t>€ 766</t>
-        </is>
-      </c>
-      <c r="F110" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="1" t="n">
-        <v>109</v>
-      </c>
-      <c r="B111" t="inlineStr">
-        <is>
-          <t>Chalet</t>
-        </is>
-      </c>
-      <c r="C111" t="n">
-        <v>4</v>
-      </c>
-      <c r="D111" t="inlineStr">
-        <is>
-          <t>€ 973</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>€ 895</t>
-        </is>
-      </c>
-      <c r="F111" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="1" t="n">
-        <v>110</v>
-      </c>
-      <c r="B112" t="inlineStr">
-        <is>
-          <t>Chalet</t>
-        </is>
-      </c>
-      <c r="C112" t="n">
-        <v>5</v>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>€ 1.043</t>
-        </is>
-      </c>
-      <c r="E112" t="inlineStr">
-        <is>
-          <t>€ 960</t>
-        </is>
-      </c>
-      <c r="F112" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G112" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="1" t="n">
-        <v>111</v>
-      </c>
-      <c r="B113" t="inlineStr">
-        <is>
-          <t>Chalet</t>
-        </is>
-      </c>
-      <c r="C113" t="n">
-        <v>6</v>
-      </c>
-      <c r="D113" t="inlineStr">
-        <is>
-          <t>€ 1.113</t>
-        </is>
-      </c>
-      <c r="E113" t="inlineStr">
-        <is>
-          <t>€ 1.024</t>
-        </is>
-      </c>
-      <c r="F113" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="114">
-      <c r="A114" s="1" t="n">
-        <v>112</v>
-      </c>
-      <c r="B114" t="inlineStr">
-        <is>
-          <t>Chalet</t>
-        </is>
-      </c>
-      <c r="C114" t="n">
-        <v>1</v>
-      </c>
-      <c r="D114" t="inlineStr">
-        <is>
-          <t>€ 413</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>€ 380</t>
-        </is>
-      </c>
-      <c r="F114" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/parco-gessilandia.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>parco-gessilandia</t>
-        </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" s="1" t="n">
-        <v>113</v>
-      </c>
-      <c r="B115" t="inlineStr">
-        <is>
-          <t>Tenda</t>
-        </is>
-      </c>
-      <c r="C115" t="n">
-        <v>4</v>
-      </c>
-      <c r="D115" t="inlineStr"/>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>€ 840</t>
-        </is>
-      </c>
-      <c r="F115" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/resort-orizzonti-glamping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>resort-orizzonti-glamping</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="1" t="n">
-        <v>114</v>
-      </c>
-      <c r="B116" t="inlineStr">
-        <is>
-          <t>Tenda</t>
-        </is>
-      </c>
-      <c r="C116" t="n">
-        <v>5</v>
-      </c>
-      <c r="D116" t="inlineStr"/>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>€ 910</t>
-        </is>
-      </c>
-      <c r="F116" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/resort-orizzonti-glamping.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>resort-orizzonti-glamping</t>
-        </is>
-      </c>
-    </row>
-    <row r="117">
-      <c r="A117" s="1" t="n">
-        <v>115</v>
-      </c>
-      <c r="B117" t="inlineStr">
-        <is>
-          <t>Roulotte</t>
-        </is>
-      </c>
-      <c r="C117" t="n">
-        <v>2</v>
-      </c>
-      <c r="D117" t="inlineStr">
-        <is>
-          <t>€ 455</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>€ 419</t>
-        </is>
-      </c>
-      <c r="F117" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/antica-dimora-campeggio-fiordaliso.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>antica-dimora-campeggio-fiordaliso</t>
-        </is>
-      </c>
-    </row>
-    <row r="118">
-      <c r="A118" s="1" t="n">
-        <v>116</v>
-      </c>
-      <c r="B118" t="inlineStr">
-        <is>
-          <t>Rifugio Safari</t>
-        </is>
-      </c>
-      <c r="C118" t="n">
-        <v>2</v>
-      </c>
-      <c r="D118" t="inlineStr">
-        <is>
-          <t>€ 779</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>€ 650</t>
-        </is>
-      </c>
-      <c r="F118" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/camping-podere-sei-poorte.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t>camping-podere-sei-poorte</t>
-        </is>
-      </c>
-    </row>
-    <row r="119">
-      <c r="A119" s="1" t="n">
-        <v>117</v>
-      </c>
-      <c r="B119" t="inlineStr">
-        <is>
-          <t>Tenda</t>
-        </is>
-      </c>
-      <c r="C119" t="n">
-        <v>2</v>
-      </c>
-      <c r="D119" t="inlineStr">
-        <is>
-          <t>€ 525</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>€ 488</t>
-        </is>
-      </c>
-      <c r="F119" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/safaritent-glamping-mar-y-sierrra.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t>safaritent-glamping-mar-y-sierrra</t>
-        </is>
-      </c>
-    </row>
-    <row r="120">
-      <c r="A120" s="1" t="n">
-        <v>118</v>
-      </c>
-      <c r="B120" t="inlineStr">
-        <is>
-          <t>Bungalow con 2 Camere da Letto (4 Adulti)</t>
-        </is>
-      </c>
-      <c r="C120" t="n">
-        <v>4</v>
-      </c>
-      <c r="D120" t="inlineStr"/>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>€ 680</t>
-        </is>
-      </c>
-      <c r="F120" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/camping-norina.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G120" t="inlineStr">
-        <is>
           <t>camping-norina</t>
-        </is>
-      </c>
-    </row>
-    <row r="121">
-      <c r="A121" s="1" t="n">
-        <v>119</v>
-      </c>
-      <c r="B121" t="inlineStr">
-        <is>
-          <t>Bungalow con 2 Camere da Letto (5 Adulti)</t>
-        </is>
-      </c>
-      <c r="C121" t="n">
-        <v>5</v>
-      </c>
-      <c r="D121" t="inlineStr"/>
-      <c r="E121" t="inlineStr">
-        <is>
-          <t>€ 785</t>
-        </is>
-      </c>
-      <c r="F121" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/camping-norina.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>camping-norina</t>
-        </is>
-      </c>
-    </row>
-    <row r="122">
-      <c r="A122" s="1" t="n">
-        <v>120</v>
-      </c>
-      <c r="B122" t="inlineStr">
-        <is>
-          <t>Cottage</t>
-        </is>
-      </c>
-      <c r="C122" t="n">
-        <v>2</v>
-      </c>
-      <c r="D122" t="inlineStr"/>
-      <c r="E122" t="inlineStr">
-        <is>
-          <t>€ 526</t>
-        </is>
-      </c>
-      <c r="F122" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/camping-paradiso.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>camping-paradiso</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="1" t="n">
-        <v>121</v>
-      </c>
-      <c r="B123" t="inlineStr">
-        <is>
-          <t>Cottage</t>
-        </is>
-      </c>
-      <c r="C123" t="n">
-        <v>3</v>
-      </c>
-      <c r="D123" t="inlineStr"/>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>€ 596</t>
-        </is>
-      </c>
-      <c r="F123" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/camping-paradiso.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>camping-paradiso</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="1" t="n">
-        <v>122</v>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>Cottage</t>
-        </is>
-      </c>
-      <c r="C124" t="n">
-        <v>4</v>
-      </c>
-      <c r="D124" t="inlineStr"/>
-      <c r="E124" t="inlineStr">
-        <is>
-          <t>€ 631</t>
-        </is>
-      </c>
-      <c r="F124" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/camping-paradiso.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>camping-paradiso</t>
-        </is>
-      </c>
-    </row>
-    <row r="125">
-      <c r="A125" s="1" t="n">
-        <v>123</v>
-      </c>
-      <c r="B125" t="inlineStr">
-        <is>
-          <t>Bungalow</t>
-        </is>
-      </c>
-      <c r="C125" t="n">
-        <v>2</v>
-      </c>
-      <c r="D125" t="inlineStr"/>
-      <c r="E125" t="inlineStr">
-        <is>
-          <t>€ 505</t>
-        </is>
-      </c>
-      <c r="F125" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/camping-pineta-urbino.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>camping-pineta-urbino</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="1" t="n">
-        <v>124</v>
-      </c>
-      <c r="B126" t="inlineStr">
-        <is>
-          <t>Bungalow</t>
-        </is>
-      </c>
-      <c r="C126" t="n">
-        <v>3</v>
-      </c>
-      <c r="D126" t="inlineStr"/>
-      <c r="E126" t="inlineStr">
-        <is>
-          <t>€ 724</t>
-        </is>
-      </c>
-      <c r="F126" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/camping-pineta-urbino.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>camping-pineta-urbino</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="1" t="n">
-        <v>125</v>
-      </c>
-      <c r="B127" t="inlineStr">
-        <is>
-          <t>Bungalow</t>
-        </is>
-      </c>
-      <c r="C127" t="n">
-        <v>4</v>
-      </c>
-      <c r="D127" t="inlineStr"/>
-      <c r="E127" t="inlineStr">
-        <is>
-          <t>€ 942</t>
-        </is>
-      </c>
-      <c r="F127" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/camping-pineta-urbino.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>camping-pineta-urbino</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" s="1" t="n">
-        <v>126</v>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>Bungalow con Vista Mare</t>
-        </is>
-      </c>
-      <c r="C128" t="n">
-        <v>5</v>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>€ 1.124</t>
-        </is>
-      </c>
-      <c r="E128" t="inlineStr">
-        <is>
-          <t>€ 1.040</t>
-        </is>
-      </c>
-      <c r="F128" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/bungalow-verde-mare.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>bungalow-verde-mare</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" s="1" t="n">
-        <v>127</v>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>Tenda</t>
-        </is>
-      </c>
-      <c r="C129" t="n">
-        <v>2</v>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>€ 464</t>
-        </is>
-      </c>
-      <c r="E129" t="inlineStr">
-        <is>
-          <t>€ 434</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/glamping-marche-nascoste-tenda-e-intero-alloggio.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>glamping-marche-nascoste-tenda-e-intero-alloggio</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="1" t="n">
-        <v>128</v>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>Tenda</t>
-        </is>
-      </c>
-      <c r="C130" t="n">
-        <v>3</v>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>€ 618</t>
-        </is>
-      </c>
-      <c r="E130" t="inlineStr">
-        <is>
-          <t>€ 578</t>
-        </is>
-      </c>
-      <c r="F130" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/glamping-marche-nascoste-tenda-e-intero-alloggio.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>glamping-marche-nascoste-tenda-e-intero-alloggio</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="1" t="n">
-        <v>129</v>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>Tenda</t>
-        </is>
-      </c>
-      <c r="C131" t="n">
-        <v>4</v>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>€ 464</t>
-        </is>
-      </c>
-      <c r="E131" t="inlineStr">
-        <is>
-          <t>€ 434</t>
-        </is>
-      </c>
-      <c r="F131" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/glamping-marche-nascoste-tenda-e-intero-alloggio.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>glamping-marche-nascoste-tenda-e-intero-alloggio</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="1" t="n">
-        <v>130</v>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>Tenda</t>
-        </is>
-      </c>
-      <c r="C132" t="n">
-        <v>4</v>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>€ 772</t>
-        </is>
-      </c>
-      <c r="E132" t="inlineStr">
-        <is>
-          <t>€ 722</t>
-        </is>
-      </c>
-      <c r="F132" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/glamping-marche-nascoste-tenda-e-intero-alloggio.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G132" t="inlineStr">
-        <is>
-          <t>glamping-marche-nascoste-tenda-e-intero-alloggio</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" s="1" t="n">
-        <v>131</v>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>Tenda</t>
-        </is>
-      </c>
-      <c r="C133" t="n">
-        <v>1</v>
-      </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>€ 429</t>
-        </is>
-      </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>€ 401</t>
-        </is>
-      </c>
-      <c r="F133" t="inlineStr">
-        <is>
-          <t>https://www.booking.com/hotel/it/glamping-marche-nascoste-tenda-e-intero-alloggio.it.html?checkin=2022-09-17;checkout=2022-09-24;selected_currency=EUR</t>
-        </is>
-      </c>
-      <c r="G133" t="inlineStr">
-        <is>
-          <t>glamping-marche-nascoste-tenda-e-intero-alloggio</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
eliminata la funzionalità che permette di prendere automaticamente i link da booking, ora i link dei camping sono passati manualmente da noi. I metodi sono comunque stati mantenuti  ma etichettati come OLD in caso dovessero tornare utili in quanto funzionanti
</commit_message>
<xml_diff>
--- a/datasets/availability_dataset_2022-09-17_2022-09-24_booking.xlsx
+++ b/datasets/availability_dataset_2022-09-17_2022-09-24_booking.xlsx
@@ -2233,7 +2233,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>€ 349</t>
+          <t>€ 344</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2266,7 +2266,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>€ 404</t>
+          <t>€ 399</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2299,7 +2299,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>€ 404</t>
+          <t>€ 399</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
@@ -2332,7 +2332,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>€ 439</t>
+          <t>€ 433</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
@@ -2365,7 +2365,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>€ 474</t>
+          <t>€ 467</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -2398,7 +2398,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>€ 489</t>
+          <t>€ 481</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>€ 404</t>
+          <t>€ 399</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2464,7 +2464,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>€ 1.250</t>
+          <t>€ 1.150</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -2490,10 +2490,14 @@
       <c r="C68" t="n">
         <v>4</v>
       </c>
-      <c r="D68" t="inlineStr"/>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>€ 1.470</t>
+        </is>
+      </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>€ 1.470</t>
+          <t>€ 1.352</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -2606,14 +2610,10 @@
       <c r="C72" t="n">
         <v>2</v>
       </c>
-      <c r="D72" t="inlineStr">
+      <c r="D72" t="inlineStr"/>
+      <c r="E72" t="inlineStr">
         <is>
           <t>€ 464</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>€ 434</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -2639,14 +2639,10 @@
       <c r="C73" t="n">
         <v>3</v>
       </c>
-      <c r="D73" t="inlineStr">
+      <c r="D73" t="inlineStr"/>
+      <c r="E73" t="inlineStr">
         <is>
           <t>€ 618</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>€ 578</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -2672,14 +2668,10 @@
       <c r="C74" t="n">
         <v>4</v>
       </c>
-      <c r="D74" t="inlineStr">
+      <c r="D74" t="inlineStr"/>
+      <c r="E74" t="inlineStr">
         <is>
           <t>€ 464</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>€ 434</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -2705,14 +2697,10 @@
       <c r="C75" t="n">
         <v>4</v>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D75" t="inlineStr"/>
+      <c r="E75" t="inlineStr">
         <is>
           <t>€ 772</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>€ 722</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
@@ -2738,14 +2726,10 @@
       <c r="C76" t="n">
         <v>1</v>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
         <is>
           <t>€ 429</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>€ 401</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
@@ -2865,7 +2849,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>€ 458</t>
+          <t>€ 451</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -2898,7 +2882,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>€ 692</t>
+          <t>€ 703</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -2931,7 +2915,7 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>€ 1.175</t>
+          <t>€ 1.193</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -2964,7 +2948,7 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>€ 1.336</t>
+          <t>€ 1.357</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -2997,7 +2981,7 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>€ 1.658</t>
+          <t>€ 1.684</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -3030,7 +3014,7 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>€ 692</t>
+          <t>€ 703</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -3063,7 +3047,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>€ 1.078</t>
+          <t>€ 1.095</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3096,7 +3080,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>€ 1.336</t>
+          <t>€ 1.357</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3129,7 +3113,7 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>€ 692</t>
+          <t>€ 703</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
@@ -3162,7 +3146,7 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>€ 563</t>
+          <t>€ 572</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
@@ -3195,7 +3179,7 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>€ 724</t>
+          <t>€ 735</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
@@ -3228,7 +3212,7 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>€ 1.175</t>
+          <t>€ 1.193</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
@@ -3261,7 +3245,7 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>€ 1.040</t>
+          <t>€ 1.093</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">

</xml_diff>